<commit_message>
arreglos en el mapeo fisico
</commit_message>
<xml_diff>
--- a/Diagrama de tablas IPC2 Proyecto 1 .xlsx
+++ b/Diagrama de tablas IPC2 Proyecto 1 .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\OneDrive\Documents\Proyecto_1_IPC2_JulioOvalle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1158DDD5-811E-4B4D-8646-CA4939F3B0F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE477F19-9385-4E40-87C8-2E28B92117C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{AC607708-AF35-4EB0-AAB4-58680187AFD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="74">
   <si>
     <t>Entidad Usuario</t>
   </si>
@@ -255,6 +255,9 @@
   </si>
   <si>
     <t>porcentaje_comision</t>
+  </si>
+  <si>
+    <t>nombre_instalacion</t>
   </si>
 </sst>
 </file>
@@ -270,7 +273,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -280,6 +283,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -324,15 +333,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,7 +697,7 @@
     <col min="9" max="9" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +711,7 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
@@ -718,7 +737,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -744,7 +763,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -770,7 +789,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -796,7 +815,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -810,7 +829,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
@@ -827,7 +846,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -853,7 +872,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -879,7 +898,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -905,7 +924,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>65</v>
       </c>
@@ -931,7 +950,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -939,7 +958,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -964,8 +983,11 @@
       <c r="I14" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>26</v>
       </c>
@@ -990,8 +1012,11 @@
       <c r="I15" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>27</v>
       </c>
@@ -1014,6 +1039,9 @@
         <v>17</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="9" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1042,6 +1070,9 @@
       <c r="I17" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="J17" s="9">
+        <v>35</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -1068,6 +1099,9 @@
       <c r="I18" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="J18" s="9" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -1094,6 +1128,9 @@
       <c r="I19" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="J19" s="9" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -1108,6 +1145,7 @@
       <c r="D20" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -1122,6 +1160,7 @@
       <c r="D21" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="J21" s="10"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
@@ -1136,43 +1175,48 @@
       <c r="D22" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="J22" s="10"/>
+    </row>
+    <row r="23" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>17</v>
+      <c r="B23" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>43</v>
       </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
       <c r="G26" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="6" t="s">
         <v>45</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -1189,19 +1233,19 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="C28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="2" t="s">
@@ -1218,19 +1262,19 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E29" s="4">
+      <c r="C29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="7">
         <v>35</v>
       </c>
       <c r="G29" s="2" t="s">
@@ -1247,19 +1291,19 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="B30" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="2" t="s">
@@ -1271,7 +1315,7 @@
       <c r="I30" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="J30" s="11" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1362,8 +1406,8 @@
       <c r="D36" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>58</v>
+      <c r="F36" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -1388,12 +1432,6 @@
       <c r="D37" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">

</xml_diff>

<commit_message>
avances en las vistas
</commit_message>
<xml_diff>
--- a/Diagrama de tablas IPC2 Proyecto 1 .xlsx
+++ b/Diagrama de tablas IPC2 Proyecto 1 .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\OneDrive\Documents\Proyecto_1_IPC2_JulioOvalle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE477F19-9385-4E40-87C8-2E28B92117C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218CEDFE-C297-42D6-AE22-4903BD9DAFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{AC607708-AF35-4EB0-AAB4-58680187AFD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="74">
   <si>
     <t>Entidad Usuario</t>
   </si>
@@ -1432,6 +1432,32 @@
       <c r="D37" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F37" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F38" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
@@ -1442,16 +1468,16 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D43" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F43" s="1" t="s">

</xml_diff>

<commit_message>
creacion del manual tecnico
</commit_message>
<xml_diff>
--- a/Diagrama de tablas IPC2 Proyecto 1 .xlsx
+++ b/Diagrama de tablas IPC2 Proyecto 1 .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\OneDrive\Documents\Proyecto_1_IPC2_JulioOvalle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218CEDFE-C297-42D6-AE22-4903BD9DAFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A621E1A0-B88C-491B-94E2-184311F7BE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{AC607708-AF35-4EB0-AAB4-58680187AFD8}"/>
   </bookViews>
@@ -273,7 +273,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -283,12 +283,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -333,25 +327,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -983,7 +974,7 @@
       <c r="I14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="4" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1012,7 +1003,7 @@
       <c r="I15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="J15" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1041,7 +1032,7 @@
       <c r="I16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="J16" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1070,7 +1061,7 @@
       <c r="I17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="5">
         <v>35</v>
       </c>
     </row>
@@ -1099,7 +1090,7 @@
       <c r="I18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="J18" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1128,7 +1119,7 @@
       <c r="I19" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="J19" s="9" t="s">
+      <c r="J19" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1145,7 +1136,6 @@
       <c r="D20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -1160,7 +1150,6 @@
       <c r="D21" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="J21" s="10"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
@@ -1175,48 +1164,47 @@
       <c r="D22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J22" s="10"/>
-    </row>
-    <row r="23" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D23" s="11" t="s">
+      <c r="B23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
       <c r="G26" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="1" t="s">
         <v>45</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -1233,19 +1221,19 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="6" t="s">
+      <c r="C28" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="2" t="s">
@@ -1262,19 +1250,19 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E29" s="7">
+      <c r="C29" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="8">
         <v>35</v>
       </c>
       <c r="G29" s="2" t="s">
@@ -1291,19 +1279,19 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E30" s="6" t="s">
+      <c r="B30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="2" t="s">
@@ -1315,7 +1303,7 @@
       <c r="I30" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J30" s="11" t="s">
+      <c r="J30" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1406,7 +1394,7 @@
       <c r="D36" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F36" s="11" t="s">
+      <c r="F36" s="2" t="s">
         <v>73</v>
       </c>
       <c r="G36" s="2" t="s">
@@ -1432,7 +1420,7 @@
       <c r="D37" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F37" s="11" t="s">
+      <c r="F37" s="2" t="s">
         <v>73</v>
       </c>
       <c r="G37" s="2" t="s">
@@ -1446,7 +1434,7 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="2" t="s">
         <v>31</v>
       </c>
       <c r="G38" s="2" t="s">

</xml_diff>